<commit_message>
docs(#298): documente le renommage IdentityReliability → IdentityStatus dans le changelog
Ajoute une entrée [BREAKING CHANGE] recensant les anciennes/nouvelles URLs
canoniques du CodeSystem et des ValueSets renommés, pour les implémenteurs
qui auraient déjà référencé les noms précédents. a3a7a24abf05f9aed5958192a646a7b66e2d7f7d
</commit_message>
<xml_diff>
--- a/fix/issue-298-identity-status-rniv/ig/StructureDefinition-fr-core-identity-reliability.xlsx
+++ b/fix/issue-298-identity-status-rniv/ig/StructureDefinition-fr-core-identity-reliability.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-07T07:47:42+00:00</t>
+    <t>2026-08-07T08:01:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -458,7 +458,7 @@
     <t>required</t>
   </si>
   <si>
-    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-identity-reliability|2.2.0</t>
+    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-identity-status|2.2.0</t>
   </si>
   <si>
     <t>Extension.extension:comment</t>
@@ -482,7 +482,7 @@
     <t>Extension.extension:comment.value[x]</t>
   </si>
   <si>
-    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-identity-reliability-supplement|2.2.0</t>
+    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-identity-status-comment|2.2.0</t>
   </si>
   <si>
     <t>Extension.extension:validationDate</t>
@@ -879,7 +879,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="18.49609375" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="64.2109375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="61.1953125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>

</xml_diff>

<commit_message>
fix: réécrit Description/purpose de fr-core-identity-reliability et retire le short racine
Corrige la faute "Reliabilility" et le texte obsolète (ne mentionnait que
2 statuts) pour refléter la structure actuelle : 4 statuts RNIV
(PROV/RECUP/VALI/QUAL), canal de collecte, pièce justificative, dates et
annotations. Supprime la ligne ^short sur l'élément racine, redondante
avec le Title.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 5d72d3189e70300b3aa65904a85047b883c52b1a
</commit_message>
<xml_diff>
--- a/fix/issue-298-identity-status-rniv/ig/StructureDefinition-fr-core-identity-reliability.xlsx
+++ b/fix/issue-298-identity-status-rniv/ig/StructureDefinition-fr-core-identity-reliability.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="168">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-10T13:45:29+00:00</t>
+    <t>2026-08-10T13:54:17+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,16 +84,15 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Précision sur le degré de fiabilité de l'identité du patient (si provisoire, validé... avec la justification : quelle type de pièce d'identité ?) accompagné de la méthode de collection.
--Reliabilility of the patient's identity</t>
+    <t>Extension composite précisant le degré de confiance de l'identité du patient au sens du Référentiel National d'Identitovigilance (RNIV) : statut de confiance (provisoire, récupérée, validée, qualifiée), canal d'obtention des traits d'identité ou de l'INS, pièce justificative contrôlée, dates associées et annotations complémentaires.
+Composite extension specifying the confidence level of a patient's identity per the French National Identity Vigilance Framework (RNIV): trust status (provisional, recovered, validated, qualified), channel used to collect the identity traits or the INS, validation evidence, related dates and additional annotations.</t>
   </si>
   <si>
     <t>Purpose</t>
   </si>
   <si>
-    <t>Permet de préciser le degré de fiabilité de l'identité du patient
-Reliabilility of the patient's identity</t>
+    <t>Permet de documenter le degré de confiance de l'identité d'un patient conformément au RNIV, ainsi que les éléments ayant permis de l'établir (canal de collecte, statut, justificatif de contrôle, annotations).
+Documents the confidence level of a patient's identity per the RNIV, along with the elements used to establish it (collection channel, status, validation evidence, annotations).</t>
   </si>
   <si>
     <t>Copyright</t>
@@ -263,9 +262,6 @@
   <si>
     <t xml:space="preserve">
 </t>
-  </si>
-  <si>
-    <t>Reliabilility of the identity | Fiabilité de l'identité</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1
@@ -1039,7 +1035,7 @@
         <v>81</v>
       </c>
       <c r="L2" t="s" s="2">
-        <v>82</v>
+        <v>9</v>
       </c>
       <c r="M2" t="s" s="2">
         <v>23</v>
@@ -1102,10 +1098,10 @@
         <v>80</v>
       </c>
       <c r="AI2" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ2" t="s" s="2">
         <v>83</v>
-      </c>
-      <c r="AJ2" t="s" s="2">
-        <v>84</v>
       </c>
       <c r="AK2" t="s" s="2">
         <v>78</v>
@@ -1113,10 +1109,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" t="s" s="2">
@@ -1127,25 +1123,25 @@
         <v>79</v>
       </c>
       <c r="G3" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H3" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I3" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J3" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K3" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="H3" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I3" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J3" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K3" t="s" s="2">
+      <c r="L3" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="L3" t="s" s="2">
+      <c r="M3" t="s" s="2">
         <v>88</v>
-      </c>
-      <c r="M3" t="s" s="2">
-        <v>89</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
@@ -1196,34 +1192,34 @@
         <v>78</v>
       </c>
       <c r="AF3" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AG3" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH3" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI3" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ3" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK3" t="s" s="2">
         <v>90</v>
-      </c>
-      <c r="AG3" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH3" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI3" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ3" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK3" t="s" s="2">
-        <v>91</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" t="s" s="2">
@@ -1242,16 +1238,16 @@
         <v>78</v>
       </c>
       <c r="K4" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="L4" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="L4" t="s" s="2">
+      <c r="M4" t="s" s="2">
         <v>95</v>
       </c>
-      <c r="M4" t="s" s="2">
+      <c r="N4" t="s" s="2">
         <v>96</v>
-      </c>
-      <c r="N4" t="s" s="2">
-        <v>97</v>
       </c>
       <c r="O4" s="2"/>
       <c r="P4" t="s" s="2">
@@ -1289,19 +1285,19 @@
         <v>78</v>
       </c>
       <c r="AB4" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AC4" t="s" s="2">
         <v>98</v>
       </c>
-      <c r="AC4" t="s" s="2">
+      <c r="AD4" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE4" t="s" s="2">
         <v>99</v>
       </c>
-      <c r="AD4" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE4" t="s" s="2">
+      <c r="AF4" t="s" s="2">
         <v>100</v>
-      </c>
-      <c r="AF4" t="s" s="2">
-        <v>101</v>
       </c>
       <c r="AG4" t="s" s="2">
         <v>79</v>
@@ -1313,21 +1309,21 @@
         <v>78</v>
       </c>
       <c r="AJ4" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AK4" t="s" s="2">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="B5" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="C5" t="s" s="2">
         <v>102</v>
-      </c>
-      <c r="B5" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="C5" t="s" s="2">
-        <v>103</v>
       </c>
       <c r="D5" t="s" s="2">
         <v>78</v>
@@ -1337,7 +1333,7 @@
         <v>79</v>
       </c>
       <c r="G5" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H5" t="s" s="2">
         <v>78</v>
@@ -1349,13 +1345,13 @@
         <v>78</v>
       </c>
       <c r="K5" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L5" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="M5" t="s" s="2">
         <v>104</v>
-      </c>
-      <c r="M5" t="s" s="2">
-        <v>105</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -1406,7 +1402,7 @@
         <v>78</v>
       </c>
       <c r="AF5" t="s" s="2">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AG5" t="s" s="2">
         <v>79</v>
@@ -1418,7 +1414,7 @@
         <v>78</v>
       </c>
       <c r="AJ5" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AK5" t="s" s="2">
         <v>78</v>
@@ -1426,10 +1422,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="B6" t="s" s="2">
         <v>106</v>
-      </c>
-      <c r="B6" t="s" s="2">
-        <v>107</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
@@ -1440,25 +1436,25 @@
         <v>79</v>
       </c>
       <c r="G6" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H6" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I6" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J6" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K6" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="H6" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I6" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J6" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K6" t="s" s="2">
+      <c r="L6" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="L6" t="s" s="2">
+      <c r="M6" t="s" s="2">
         <v>88</v>
-      </c>
-      <c r="M6" t="s" s="2">
-        <v>89</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
@@ -1509,30 +1505,30 @@
         <v>78</v>
       </c>
       <c r="AF6" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AG6" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH6" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI6" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ6" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK6" t="s" s="2">
         <v>90</v>
-      </c>
-      <c r="AG6" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH6" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI6" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ6" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK6" t="s" s="2">
-        <v>91</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="B7" t="s" s="2">
         <v>108</v>
-      </c>
-      <c r="B7" t="s" s="2">
-        <v>109</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
@@ -1555,13 +1551,13 @@
         <v>78</v>
       </c>
       <c r="K7" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L7" t="s" s="2">
         <v>32</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1600,19 +1596,19 @@
         <v>78</v>
       </c>
       <c r="AB7" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AC7" t="s" s="2">
         <v>98</v>
       </c>
-      <c r="AC7" t="s" s="2">
+      <c r="AD7" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE7" t="s" s="2">
         <v>99</v>
       </c>
-      <c r="AD7" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE7" t="s" s="2">
+      <c r="AF7" t="s" s="2">
         <v>100</v>
-      </c>
-      <c r="AF7" t="s" s="2">
-        <v>101</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>79</v>
@@ -1624,7 +1620,7 @@
         <v>78</v>
       </c>
       <c r="AJ7" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AK7" t="s" s="2">
         <v>78</v>
@@ -1632,10 +1628,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="B8" t="s" s="2">
         <v>111</v>
-      </c>
-      <c r="B8" t="s" s="2">
-        <v>112</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1643,10 +1639,10 @@
       </c>
       <c r="E8" s="2"/>
       <c r="F8" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G8" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H8" t="s" s="2">
         <v>78</v>
@@ -1658,16 +1654,16 @@
         <v>78</v>
       </c>
       <c r="K8" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="L8" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="L8" t="s" s="2">
+      <c r="M8" t="s" s="2">
         <v>114</v>
       </c>
-      <c r="M8" t="s" s="2">
+      <c r="N8" t="s" s="2">
         <v>115</v>
-      </c>
-      <c r="N8" t="s" s="2">
-        <v>116</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" t="s" s="2">
@@ -1675,7 +1671,7 @@
       </c>
       <c r="Q8" s="2"/>
       <c r="R8" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="S8" t="s" s="2">
         <v>78</v>
@@ -1717,30 +1713,30 @@
         <v>78</v>
       </c>
       <c r="AF8" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AG8" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AH8" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI8" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ8" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK8" t="s" s="2">
         <v>117</v>
-      </c>
-      <c r="AG8" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AH8" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI8" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ8" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK8" t="s" s="2">
-        <v>118</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="B9" t="s" s="2">
         <v>119</v>
-      </c>
-      <c r="B9" t="s" s="2">
-        <v>120</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -1751,7 +1747,7 @@
         <v>79</v>
       </c>
       <c r="G9" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H9" t="s" s="2">
         <v>78</v>
@@ -1763,13 +1759,13 @@
         <v>78</v>
       </c>
       <c r="K9" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="L9" t="s" s="2">
         <v>121</v>
       </c>
-      <c r="L9" t="s" s="2">
+      <c r="M9" t="s" s="2">
         <v>122</v>
-      </c>
-      <c r="M9" t="s" s="2">
-        <v>123</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -1796,55 +1792,55 @@
         <v>78</v>
       </c>
       <c r="X9" t="s" s="2">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="Y9" s="2"/>
       <c r="Z9" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="AA9" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB9" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC9" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD9" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE9" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF9" t="s" s="2">
         <v>125</v>
       </c>
-      <c r="AA9" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB9" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC9" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD9" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE9" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF9" t="s" s="2">
+      <c r="AG9" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH9" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI9" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ9" t="s" s="2">
         <v>126</v>
       </c>
-      <c r="AG9" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH9" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI9" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ9" t="s" s="2">
-        <v>127</v>
-      </c>
       <c r="AK9" t="s" s="2">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
+        <v>127</v>
+      </c>
+      <c r="B10" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="C10" t="s" s="2">
         <v>128</v>
-      </c>
-      <c r="B10" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="C10" t="s" s="2">
-        <v>129</v>
       </c>
       <c r="D10" t="s" s="2">
         <v>78</v>
@@ -1854,7 +1850,7 @@
         <v>79</v>
       </c>
       <c r="G10" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H10" t="s" s="2">
         <v>78</v>
@@ -1866,13 +1862,13 @@
         <v>78</v>
       </c>
       <c r="K10" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -1923,7 +1919,7 @@
         <v>78</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>79</v>
@@ -1935,7 +1931,7 @@
         <v>78</v>
       </c>
       <c r="AJ10" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AK10" t="s" s="2">
         <v>78</v>
@@ -1943,10 +1939,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -1957,25 +1953,25 @@
         <v>79</v>
       </c>
       <c r="G11" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H11" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I11" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J11" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K11" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="H11" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I11" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J11" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K11" t="s" s="2">
+      <c r="L11" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="L11" t="s" s="2">
+      <c r="M11" t="s" s="2">
         <v>88</v>
-      </c>
-      <c r="M11" t="s" s="2">
-        <v>89</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -2026,30 +2022,30 @@
         <v>78</v>
       </c>
       <c r="AF11" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AG11" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH11" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI11" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ11" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK11" t="s" s="2">
         <v>90</v>
-      </c>
-      <c r="AG11" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH11" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI11" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ11" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK11" t="s" s="2">
-        <v>91</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2072,13 +2068,13 @@
         <v>78</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L12" t="s" s="2">
         <v>32</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -2117,19 +2113,19 @@
         <v>78</v>
       </c>
       <c r="AB12" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AC12" t="s" s="2">
         <v>98</v>
       </c>
-      <c r="AC12" t="s" s="2">
+      <c r="AD12" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE12" t="s" s="2">
         <v>99</v>
       </c>
-      <c r="AD12" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE12" t="s" s="2">
+      <c r="AF12" t="s" s="2">
         <v>100</v>
-      </c>
-      <c r="AF12" t="s" s="2">
-        <v>101</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>79</v>
@@ -2141,7 +2137,7 @@
         <v>78</v>
       </c>
       <c r="AJ12" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AK12" t="s" s="2">
         <v>78</v>
@@ -2149,10 +2145,10 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2160,10 +2156,10 @@
       </c>
       <c r="E13" s="2"/>
       <c r="F13" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G13" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H13" t="s" s="2">
         <v>78</v>
@@ -2175,16 +2171,16 @@
         <v>78</v>
       </c>
       <c r="K13" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="L13" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="L13" t="s" s="2">
+      <c r="M13" t="s" s="2">
         <v>114</v>
       </c>
-      <c r="M13" t="s" s="2">
+      <c r="N13" t="s" s="2">
         <v>115</v>
-      </c>
-      <c r="N13" t="s" s="2">
-        <v>116</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -2192,7 +2188,7 @@
       </c>
       <c r="Q13" s="2"/>
       <c r="R13" t="s" s="2">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="S13" t="s" s="2">
         <v>78</v>
@@ -2234,30 +2230,30 @@
         <v>78</v>
       </c>
       <c r="AF13" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AG13" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AH13" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI13" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ13" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK13" t="s" s="2">
         <v>117</v>
-      </c>
-      <c r="AG13" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AH13" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI13" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ13" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK13" t="s" s="2">
-        <v>118</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2268,7 +2264,7 @@
         <v>79</v>
       </c>
       <c r="G14" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H14" t="s" s="2">
         <v>78</v>
@@ -2280,13 +2276,13 @@
         <v>78</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="L14" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="M14" t="s" s="2">
         <v>122</v>
-      </c>
-      <c r="M14" t="s" s="2">
-        <v>123</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2337,33 +2333,33 @@
         <v>78</v>
       </c>
       <c r="AF14" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="AG14" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH14" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI14" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ14" t="s" s="2">
         <v>126</v>
       </c>
-      <c r="AG14" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH14" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI14" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ14" t="s" s="2">
-        <v>127</v>
-      </c>
       <c r="AK14" t="s" s="2">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="B15" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="C15" t="s" s="2">
         <v>136</v>
-      </c>
-      <c r="B15" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="C15" t="s" s="2">
-        <v>137</v>
       </c>
       <c r="D15" t="s" s="2">
         <v>78</v>
@@ -2373,7 +2369,7 @@
         <v>79</v>
       </c>
       <c r="G15" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H15" t="s" s="2">
         <v>78</v>
@@ -2385,13 +2381,13 @@
         <v>78</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2442,7 +2438,7 @@
         <v>78</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>79</v>
@@ -2454,7 +2450,7 @@
         <v>78</v>
       </c>
       <c r="AJ15" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AK15" t="s" s="2">
         <v>78</v>
@@ -2462,10 +2458,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2476,25 +2472,25 @@
         <v>79</v>
       </c>
       <c r="G16" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H16" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I16" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J16" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K16" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="H16" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I16" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J16" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K16" t="s" s="2">
+      <c r="L16" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="L16" t="s" s="2">
+      <c r="M16" t="s" s="2">
         <v>88</v>
-      </c>
-      <c r="M16" t="s" s="2">
-        <v>89</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -2545,30 +2541,30 @@
         <v>78</v>
       </c>
       <c r="AF16" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AG16" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH16" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI16" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ16" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK16" t="s" s="2">
         <v>90</v>
-      </c>
-      <c r="AG16" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH16" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI16" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ16" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK16" t="s" s="2">
-        <v>91</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -2591,13 +2587,13 @@
         <v>78</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L17" t="s" s="2">
         <v>32</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -2636,19 +2632,19 @@
         <v>78</v>
       </c>
       <c r="AB17" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AC17" t="s" s="2">
         <v>98</v>
       </c>
-      <c r="AC17" t="s" s="2">
+      <c r="AD17" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE17" t="s" s="2">
         <v>99</v>
       </c>
-      <c r="AD17" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE17" t="s" s="2">
+      <c r="AF17" t="s" s="2">
         <v>100</v>
-      </c>
-      <c r="AF17" t="s" s="2">
-        <v>101</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>79</v>
@@ -2660,7 +2656,7 @@
         <v>78</v>
       </c>
       <c r="AJ17" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AK17" t="s" s="2">
         <v>78</v>
@@ -2668,10 +2664,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -2679,10 +2675,10 @@
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G18" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H18" t="s" s="2">
         <v>78</v>
@@ -2694,16 +2690,16 @@
         <v>78</v>
       </c>
       <c r="K18" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="L18" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="L18" t="s" s="2">
+      <c r="M18" t="s" s="2">
         <v>114</v>
       </c>
-      <c r="M18" t="s" s="2">
+      <c r="N18" t="s" s="2">
         <v>115</v>
-      </c>
-      <c r="N18" t="s" s="2">
-        <v>116</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -2711,7 +2707,7 @@
       </c>
       <c r="Q18" s="2"/>
       <c r="R18" t="s" s="2">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="S18" t="s" s="2">
         <v>78</v>
@@ -2753,30 +2749,30 @@
         <v>78</v>
       </c>
       <c r="AF18" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AG18" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AH18" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI18" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ18" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK18" t="s" s="2">
         <v>117</v>
-      </c>
-      <c r="AG18" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AH18" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI18" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ18" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK18" t="s" s="2">
-        <v>118</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -2787,7 +2783,7 @@
         <v>79</v>
       </c>
       <c r="G19" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H19" t="s" s="2">
         <v>78</v>
@@ -2799,13 +2795,13 @@
         <v>78</v>
       </c>
       <c r="K19" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="L19" t="s" s="2">
         <v>121</v>
       </c>
-      <c r="L19" t="s" s="2">
+      <c r="M19" t="s" s="2">
         <v>122</v>
-      </c>
-      <c r="M19" t="s" s="2">
-        <v>123</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -2832,11 +2828,11 @@
         <v>78</v>
       </c>
       <c r="X19" t="s" s="2">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="Y19" s="2"/>
       <c r="Z19" t="s" s="2">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AA19" t="s" s="2">
         <v>78</v>
@@ -2854,33 +2850,33 @@
         <v>78</v>
       </c>
       <c r="AF19" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="AG19" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH19" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI19" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ19" t="s" s="2">
         <v>126</v>
       </c>
-      <c r="AG19" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH19" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI19" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ19" t="s" s="2">
-        <v>127</v>
-      </c>
       <c r="AK19" t="s" s="2">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="B20" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="C20" t="s" s="2">
         <v>145</v>
-      </c>
-      <c r="B20" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="C20" t="s" s="2">
-        <v>146</v>
       </c>
       <c r="D20" t="s" s="2">
         <v>78</v>
@@ -2902,13 +2898,13 @@
         <v>78</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -2959,7 +2955,7 @@
         <v>78</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>79</v>
@@ -2971,7 +2967,7 @@
         <v>78</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AK20" t="s" s="2">
         <v>78</v>
@@ -2979,10 +2975,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -2993,25 +2989,25 @@
         <v>79</v>
       </c>
       <c r="G21" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H21" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I21" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J21" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K21" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="H21" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I21" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J21" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K21" t="s" s="2">
+      <c r="L21" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="L21" t="s" s="2">
+      <c r="M21" t="s" s="2">
         <v>88</v>
-      </c>
-      <c r="M21" t="s" s="2">
-        <v>89</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -3062,30 +3058,30 @@
         <v>78</v>
       </c>
       <c r="AF21" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AG21" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH21" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI21" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ21" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK21" t="s" s="2">
         <v>90</v>
-      </c>
-      <c r="AG21" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH21" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI21" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ21" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK21" t="s" s="2">
-        <v>91</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3108,13 +3104,13 @@
         <v>78</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L22" t="s" s="2">
         <v>32</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -3153,19 +3149,19 @@
         <v>78</v>
       </c>
       <c r="AB22" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AC22" t="s" s="2">
         <v>98</v>
       </c>
-      <c r="AC22" t="s" s="2">
+      <c r="AD22" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE22" t="s" s="2">
         <v>99</v>
       </c>
-      <c r="AD22" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE22" t="s" s="2">
+      <c r="AF22" t="s" s="2">
         <v>100</v>
-      </c>
-      <c r="AF22" t="s" s="2">
-        <v>101</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>79</v>
@@ -3177,7 +3173,7 @@
         <v>78</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AK22" t="s" s="2">
         <v>78</v>
@@ -3185,10 +3181,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3196,10 +3192,10 @@
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G23" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H23" t="s" s="2">
         <v>78</v>
@@ -3211,16 +3207,16 @@
         <v>78</v>
       </c>
       <c r="K23" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="L23" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="L23" t="s" s="2">
+      <c r="M23" t="s" s="2">
         <v>114</v>
       </c>
-      <c r="M23" t="s" s="2">
+      <c r="N23" t="s" s="2">
         <v>115</v>
-      </c>
-      <c r="N23" t="s" s="2">
-        <v>116</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -3228,7 +3224,7 @@
       </c>
       <c r="Q23" s="2"/>
       <c r="R23" t="s" s="2">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="S23" t="s" s="2">
         <v>78</v>
@@ -3270,30 +3266,30 @@
         <v>78</v>
       </c>
       <c r="AF23" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AG23" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AH23" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI23" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ23" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK23" t="s" s="2">
         <v>117</v>
-      </c>
-      <c r="AG23" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AH23" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI23" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ23" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK23" t="s" s="2">
-        <v>118</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3304,7 +3300,7 @@
         <v>79</v>
       </c>
       <c r="G24" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H24" t="s" s="2">
         <v>78</v>
@@ -3316,13 +3312,13 @@
         <v>78</v>
       </c>
       <c r="K24" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="L24" t="s" s="2">
         <v>121</v>
       </c>
-      <c r="L24" t="s" s="2">
+      <c r="M24" t="s" s="2">
         <v>122</v>
-      </c>
-      <c r="M24" t="s" s="2">
-        <v>123</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -3349,11 +3345,11 @@
         <v>78</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="Y24" s="2"/>
       <c r="Z24" t="s" s="2">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>78</v>
@@ -3371,33 +3367,33 @@
         <v>78</v>
       </c>
       <c r="AF24" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="AG24" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH24" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI24" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ24" t="s" s="2">
         <v>126</v>
       </c>
-      <c r="AG24" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH24" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI24" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ24" t="s" s="2">
-        <v>127</v>
-      </c>
       <c r="AK24" t="s" s="2">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="B25" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="C25" t="s" s="2">
         <v>153</v>
-      </c>
-      <c r="B25" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="C25" t="s" s="2">
-        <v>154</v>
       </c>
       <c r="D25" t="s" s="2">
         <v>78</v>
@@ -3407,7 +3403,7 @@
         <v>79</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>78</v>
@@ -3419,13 +3415,13 @@
         <v>78</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -3476,7 +3472,7 @@
         <v>78</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>79</v>
@@ -3488,7 +3484,7 @@
         <v>78</v>
       </c>
       <c r="AJ25" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AK25" t="s" s="2">
         <v>78</v>
@@ -3496,10 +3492,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -3510,25 +3506,25 @@
         <v>79</v>
       </c>
       <c r="G26" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H26" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I26" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J26" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K26" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="H26" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I26" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J26" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K26" t="s" s="2">
+      <c r="L26" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="L26" t="s" s="2">
+      <c r="M26" t="s" s="2">
         <v>88</v>
-      </c>
-      <c r="M26" t="s" s="2">
-        <v>89</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
@@ -3579,30 +3575,30 @@
         <v>78</v>
       </c>
       <c r="AF26" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AG26" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH26" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI26" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ26" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK26" t="s" s="2">
         <v>90</v>
-      </c>
-      <c r="AG26" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH26" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI26" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ26" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK26" t="s" s="2">
-        <v>91</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -3625,13 +3621,13 @@
         <v>78</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L27" t="s" s="2">
         <v>32</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -3670,19 +3666,19 @@
         <v>78</v>
       </c>
       <c r="AB27" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AC27" t="s" s="2">
         <v>98</v>
       </c>
-      <c r="AC27" t="s" s="2">
+      <c r="AD27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE27" t="s" s="2">
         <v>99</v>
       </c>
-      <c r="AD27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE27" t="s" s="2">
+      <c r="AF27" t="s" s="2">
         <v>100</v>
-      </c>
-      <c r="AF27" t="s" s="2">
-        <v>101</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>79</v>
@@ -3694,7 +3690,7 @@
         <v>78</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AK27" t="s" s="2">
         <v>78</v>
@@ -3702,10 +3698,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -3713,10 +3709,10 @@
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H28" t="s" s="2">
         <v>78</v>
@@ -3728,16 +3724,16 @@
         <v>78</v>
       </c>
       <c r="K28" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="L28" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="L28" t="s" s="2">
+      <c r="M28" t="s" s="2">
         <v>114</v>
       </c>
-      <c r="M28" t="s" s="2">
+      <c r="N28" t="s" s="2">
         <v>115</v>
-      </c>
-      <c r="N28" t="s" s="2">
-        <v>116</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -3745,7 +3741,7 @@
       </c>
       <c r="Q28" s="2"/>
       <c r="R28" t="s" s="2">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="S28" t="s" s="2">
         <v>78</v>
@@ -3787,30 +3783,30 @@
         <v>78</v>
       </c>
       <c r="AF28" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AG28" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AH28" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI28" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ28" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK28" t="s" s="2">
         <v>117</v>
-      </c>
-      <c r="AG28" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AH28" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI28" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ28" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK28" t="s" s="2">
-        <v>118</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -3821,7 +3817,7 @@
         <v>79</v>
       </c>
       <c r="G29" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H29" t="s" s="2">
         <v>78</v>
@@ -3833,13 +3829,13 @@
         <v>78</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="L29" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="M29" t="s" s="2">
         <v>122</v>
-      </c>
-      <c r="M29" t="s" s="2">
-        <v>123</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -3890,33 +3886,33 @@
         <v>78</v>
       </c>
       <c r="AF29" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="AG29" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH29" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI29" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ29" t="s" s="2">
         <v>126</v>
       </c>
-      <c r="AG29" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH29" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI29" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ29" t="s" s="2">
-        <v>127</v>
-      </c>
       <c r="AK29" t="s" s="2">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
+        <v>159</v>
+      </c>
+      <c r="B30" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="C30" t="s" s="2">
         <v>160</v>
-      </c>
-      <c r="B30" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="C30" t="s" s="2">
-        <v>161</v>
       </c>
       <c r="D30" t="s" s="2">
         <v>78</v>
@@ -3926,7 +3922,7 @@
         <v>79</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>78</v>
@@ -3938,13 +3934,13 @@
         <v>78</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -3995,7 +3991,7 @@
         <v>78</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>79</v>
@@ -4007,7 +4003,7 @@
         <v>78</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AK30" t="s" s="2">
         <v>78</v>
@@ -4015,10 +4011,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4029,25 +4025,25 @@
         <v>79</v>
       </c>
       <c r="G31" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H31" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I31" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J31" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K31" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="H31" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I31" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J31" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K31" t="s" s="2">
+      <c r="L31" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="L31" t="s" s="2">
+      <c r="M31" t="s" s="2">
         <v>88</v>
-      </c>
-      <c r="M31" t="s" s="2">
-        <v>89</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -4098,30 +4094,30 @@
         <v>78</v>
       </c>
       <c r="AF31" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AG31" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH31" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI31" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ31" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK31" t="s" s="2">
         <v>90</v>
-      </c>
-      <c r="AG31" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH31" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI31" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ31" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK31" t="s" s="2">
-        <v>91</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -4144,13 +4140,13 @@
         <v>78</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L32" t="s" s="2">
         <v>32</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -4189,19 +4185,19 @@
         <v>78</v>
       </c>
       <c r="AB32" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AC32" t="s" s="2">
         <v>98</v>
       </c>
-      <c r="AC32" t="s" s="2">
+      <c r="AD32" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE32" t="s" s="2">
         <v>99</v>
       </c>
-      <c r="AD32" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE32" t="s" s="2">
+      <c r="AF32" t="s" s="2">
         <v>100</v>
-      </c>
-      <c r="AF32" t="s" s="2">
-        <v>101</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>79</v>
@@ -4213,7 +4209,7 @@
         <v>78</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AK32" t="s" s="2">
         <v>78</v>
@@ -4221,10 +4217,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -4232,10 +4228,10 @@
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>78</v>
@@ -4247,16 +4243,16 @@
         <v>78</v>
       </c>
       <c r="K33" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="L33" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="L33" t="s" s="2">
+      <c r="M33" t="s" s="2">
         <v>114</v>
       </c>
-      <c r="M33" t="s" s="2">
+      <c r="N33" t="s" s="2">
         <v>115</v>
-      </c>
-      <c r="N33" t="s" s="2">
-        <v>116</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
@@ -4264,7 +4260,7 @@
       </c>
       <c r="Q33" s="2"/>
       <c r="R33" t="s" s="2">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="S33" t="s" s="2">
         <v>78</v>
@@ -4306,30 +4302,30 @@
         <v>78</v>
       </c>
       <c r="AF33" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AG33" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AH33" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI33" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ33" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK33" t="s" s="2">
         <v>117</v>
-      </c>
-      <c r="AG33" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AH33" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI33" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ33" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK33" t="s" s="2">
-        <v>118</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -4340,7 +4336,7 @@
         <v>79</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H34" t="s" s="2">
         <v>78</v>
@@ -4352,13 +4348,13 @@
         <v>78</v>
       </c>
       <c r="K34" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="L34" t="s" s="2">
         <v>121</v>
       </c>
-      <c r="L34" t="s" s="2">
+      <c r="M34" t="s" s="2">
         <v>122</v>
-      </c>
-      <c r="M34" t="s" s="2">
-        <v>123</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -4385,11 +4381,11 @@
         <v>78</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="Y34" s="2"/>
       <c r="Z34" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>78</v>
@@ -4407,30 +4403,30 @@
         <v>78</v>
       </c>
       <c r="AF34" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="AG34" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH34" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI34" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ34" t="s" s="2">
         <v>126</v>
       </c>
-      <c r="AG34" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH34" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI34" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ34" t="s" s="2">
-        <v>127</v>
-      </c>
       <c r="AK34" t="s" s="2">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -4438,10 +4434,10 @@
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H35" t="s" s="2">
         <v>78</v>
@@ -4453,16 +4449,16 @@
         <v>78</v>
       </c>
       <c r="K35" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="L35" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="L35" t="s" s="2">
+      <c r="M35" t="s" s="2">
         <v>114</v>
       </c>
-      <c r="M35" t="s" s="2">
+      <c r="N35" t="s" s="2">
         <v>115</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>116</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -4512,30 +4508,30 @@
         <v>78</v>
       </c>
       <c r="AF35" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="AG35" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AH35" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI35" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ35" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK35" t="s" s="2">
         <v>117</v>
-      </c>
-      <c r="AG35" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AH35" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI35" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ35" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK35" t="s" s="2">
-        <v>118</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -4558,13 +4554,13 @@
         <v>78</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="L36" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="M36" t="s" s="2">
         <v>122</v>
-      </c>
-      <c r="M36" t="s" s="2">
-        <v>123</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -4615,22 +4611,22 @@
         <v>78</v>
       </c>
       <c r="AF36" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="AG36" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH36" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI36" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ36" t="s" s="2">
         <v>126</v>
       </c>
-      <c r="AG36" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH36" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="AI36" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ36" t="s" s="2">
-        <v>127</v>
-      </c>
       <c r="AK36" t="s" s="2">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix dateCollection/validationDate wording and allow CodeableConcept on comment
dateCollection incorrectly restricted its short/definition to INSi
teleservice interrogation, while methodCollection allows other
collection channels. validationDate short/definition completed to
match. comment.value[x] now allows CodeableConcept in addition to
Coding to support free text.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 4abc2e7a9e06f86c8b67f8c51463ccee37519a3d
</commit_message>
<xml_diff>
--- a/fix/issue-298-identity-status-rniv/ig/StructureDefinition-fr-core-identity-reliability.xlsx
+++ b/fix/issue-298-identity-status-rniv/ig/StructureDefinition-fr-core-identity-reliability.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="171">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-10T13:54:17+00:00</t>
+    <t>2026-08-10T14:12:55+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -414,7 +414,10 @@
     <t>dateCollection</t>
   </si>
   <si>
-    <t>INS collection date| date d'interrogation du téléservice INSi</t>
+    <t>Date d'obtention des traits d'identité ou de l'INS | Date the identity traits or the INS were collected</t>
+  </si>
+  <si>
+    <t>Date à laquelle les traits d'identité ou l'INS ont été obtenus, quel que soit le canal utilisé (cf. sous-extension `methodCollection`) : saisie manuelle, lecture de la carte Vitale, interrogation directe du téléservice INSi, scan d'un code à barre/Datamatrix, lecture RFID. Cette date ne doit pas être confondue avec la date de vérification de l'identité (cf. sous-extension `validationDate`). | Date at which the identity traits or the INS were obtained, regardless of the channel used (see the `methodCollection` sub-extension): manual entry, Vitale card reading, direct query of the INSi teleservice, barcode/Datamatrix scan, RFID reading. This date must not be confused with the identity verification date (see the `validationDate` sub-extension).</t>
   </si>
   <si>
     <t>Extension.extension:dateCollection.id</t>
@@ -481,6 +484,10 @@
     <t>Extension.extension:comment.value[x]</t>
   </si>
   <si>
+    <t xml:space="preserve">CodeableConcept
+</t>
+  </si>
+  <si>
     <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-identity-status-comment|2.2.0</t>
   </si>
   <si>
@@ -490,7 +497,10 @@
     <t>validationDate</t>
   </si>
   <si>
-    <t>Date de vérification de l'identité</t>
+    <t>Date de vérification de l'identité | Identity verification date</t>
+  </si>
+  <si>
+    <t>Date à laquelle l'identité a été vérifiée sur la base de la pièce justificative contrôlée (cf. sous-extension `validationMode`). | Date at which the identity was verified based on the checked supporting document (see the `validationMode` sub-extension).</t>
   </si>
   <si>
     <t>Extension.extension:validationDate.id</t>
@@ -1868,7 +1878,7 @@
         <v>129</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -1939,7 +1949,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B11" t="s" s="2">
         <v>106</v>
@@ -2042,7 +2052,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B12" t="s" s="2">
         <v>108</v>
@@ -2145,7 +2155,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B13" t="s" s="2">
         <v>111</v>
@@ -2250,7 +2260,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B14" t="s" s="2">
         <v>119</v>
@@ -2276,7 +2286,7 @@
         <v>78</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L14" t="s" s="2">
         <v>121</v>
@@ -2353,13 +2363,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B15" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D15" t="s" s="2">
         <v>78</v>
@@ -2384,7 +2394,7 @@
         <v>93</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M15" t="s" s="2">
         <v>109</v>
@@ -2458,7 +2468,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B16" t="s" s="2">
         <v>106</v>
@@ -2561,7 +2571,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B17" t="s" s="2">
         <v>108</v>
@@ -2664,7 +2674,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B18" t="s" s="2">
         <v>111</v>
@@ -2707,7 +2717,7 @@
       </c>
       <c r="Q18" s="2"/>
       <c r="R18" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="S18" t="s" s="2">
         <v>78</v>
@@ -2769,7 +2779,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B19" t="s" s="2">
         <v>119</v>
@@ -2828,11 +2838,11 @@
         <v>78</v>
       </c>
       <c r="X19" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="Y19" s="2"/>
       <c r="Z19" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="AA19" t="s" s="2">
         <v>78</v>
@@ -2870,13 +2880,13 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B20" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C20" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D20" t="s" s="2">
         <v>78</v>
@@ -2901,7 +2911,7 @@
         <v>93</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="M20" t="s" s="2">
         <v>109</v>
@@ -2975,7 +2985,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B21" t="s" s="2">
         <v>106</v>
@@ -3078,7 +3088,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B22" t="s" s="2">
         <v>108</v>
@@ -3181,7 +3191,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B23" t="s" s="2">
         <v>111</v>
@@ -3224,7 +3234,7 @@
       </c>
       <c r="Q23" s="2"/>
       <c r="R23" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="S23" t="s" s="2">
         <v>78</v>
@@ -3286,7 +3296,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B24" t="s" s="2">
         <v>119</v>
@@ -3312,7 +3322,7 @@
         <v>78</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>120</v>
+        <v>152</v>
       </c>
       <c r="L24" t="s" s="2">
         <v>121</v>
@@ -3349,7 +3359,7 @@
       </c>
       <c r="Y24" s="2"/>
       <c r="Z24" t="s" s="2">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>78</v>
@@ -3387,13 +3397,13 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B25" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C25" t="s" s="2">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D25" t="s" s="2">
         <v>78</v>
@@ -3418,10 +3428,10 @@
         <v>93</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>109</v>
+        <v>157</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -3492,7 +3502,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B26" t="s" s="2">
         <v>106</v>
@@ -3595,7 +3605,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B27" t="s" s="2">
         <v>108</v>
@@ -3698,7 +3708,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B28" t="s" s="2">
         <v>111</v>
@@ -3741,7 +3751,7 @@
       </c>
       <c r="Q28" s="2"/>
       <c r="R28" t="s" s="2">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="S28" t="s" s="2">
         <v>78</v>
@@ -3803,7 +3813,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B29" t="s" s="2">
         <v>119</v>
@@ -3829,7 +3839,7 @@
         <v>78</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L29" t="s" s="2">
         <v>121</v>
@@ -3906,13 +3916,13 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B30" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C30" t="s" s="2">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D30" t="s" s="2">
         <v>78</v>
@@ -3937,7 +3947,7 @@
         <v>93</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="M30" t="s" s="2">
         <v>109</v>
@@ -4011,7 +4021,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B31" t="s" s="2">
         <v>106</v>
@@ -4114,7 +4124,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B32" t="s" s="2">
         <v>108</v>
@@ -4217,7 +4227,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B33" t="s" s="2">
         <v>111</v>
@@ -4260,7 +4270,7 @@
       </c>
       <c r="Q33" s="2"/>
       <c r="R33" t="s" s="2">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="S33" t="s" s="2">
         <v>78</v>
@@ -4322,7 +4332,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B34" t="s" s="2">
         <v>119</v>
@@ -4381,11 +4391,11 @@
         <v>78</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="Y34" s="2"/>
       <c r="Z34" t="s" s="2">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>78</v>
@@ -4554,7 +4564,7 @@
         <v>78</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="L36" t="s" s="2">
         <v>121</v>

</xml_diff>

<commit_message>
Fix INS vs matricule INS terminology across identity-reliability extension
"INS" designates the identity as a whole (matricule + 5 traits), not
the numeric identifier alone. Several short/definition/intro texts
coordinated "identity traits or the INS" as if INS meant just the
number, which is inaccurate — replaced with "matricule INS" / "INS
identifier" throughout, matching existing project usage. Also
resynced the dateCollection row in the intro table, which still
described the old (already-fixed) INSi-interrogation wording.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 6ccfaa9642a79f090357b4ec77aca083ce46dd13
</commit_message>
<xml_diff>
--- a/fix/issue-298-identity-status-rniv/ig/StructureDefinition-fr-core-identity-reliability.xlsx
+++ b/fix/issue-298-identity-status-rniv/ig/StructureDefinition-fr-core-identity-reliability.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-10T14:12:55+00:00</t>
+    <t>2026-08-10T14:29:18+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,8 +84,8 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Extension composite précisant le degré de confiance de l'identité du patient au sens du Référentiel National d'Identitovigilance (RNIV) : statut de confiance (provisoire, récupérée, validée, qualifiée), canal d'obtention des traits d'identité ou de l'INS, pièce justificative contrôlée, dates associées et annotations complémentaires.
-Composite extension specifying the confidence level of a patient's identity per the French National Identity Vigilance Framework (RNIV): trust status (provisional, recovered, validated, qualified), channel used to collect the identity traits or the INS, validation evidence, related dates and additional annotations.</t>
+    <t>Extension composite précisant le degré de confiance de l'identité du patient au sens du Référentiel National d'Identitovigilance (RNIV) : statut de confiance (provisoire, récupérée, validée, qualifiée), canal d'obtention des traits d'identité ou du matricule INS, pièce justificative contrôlée, dates associées et annotations complémentaires.
+Composite extension specifying the confidence level of a patient's identity per the French National Identity Vigilance Framework (RNIV): trust status (provisional, recovered, validated, qualified), channel used to collect the identity traits or the INS identifier, validation evidence, related dates and additional annotations.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -333,10 +333,10 @@
     <t>methodCollection</t>
   </si>
   <si>
-    <t>Canal d'obtention des traits d'identité ou de l'INS (SM, CV, INSi, CB, RFID, AV) | Channel used to collect the identity traits or the INS</t>
-  </si>
-  <si>
-    <t>Précise le canal par lequel les traits d'identité ou l'INS ont été obtenus : saisie manuelle, lecture de la carte Vitale, interrogation directe du téléservice INSi, scan d'un code à barre/Datamatrix, lecture RFID ou Application carte Vitale. Ce champ ne porte pas le statut de confiance résultant (cf. sous-extension `identityStatus`) ni la pièce justificative contrôlée (cf. sous-extension `validationMode`).</t>
+    <t>Canal d'obtention des traits d'identité ou du matricule INS (SM, CV, INSi, CB, RFID, AV) | Channel used to collect the identity traits or the INS identifier</t>
+  </si>
+  <si>
+    <t>Précise le canal par lequel les traits d'identité ou le matricule INS ont été obtenus : saisie manuelle, lecture de la carte Vitale, interrogation directe du téléservice INSi, scan d'un code à barre/Datamatrix, lecture RFID ou Application carte Vitale. Ce champ ne porte pas le statut de confiance résultant (cf. sous-extension `identityStatus`) ni la pièce justificative contrôlée (cf. sous-extension `validationMode`).</t>
   </si>
   <si>
     <t>Extension.extension:methodCollection.id</t>
@@ -414,10 +414,10 @@
     <t>dateCollection</t>
   </si>
   <si>
-    <t>Date d'obtention des traits d'identité ou de l'INS | Date the identity traits or the INS were collected</t>
-  </si>
-  <si>
-    <t>Date à laquelle les traits d'identité ou l'INS ont été obtenus, quel que soit le canal utilisé (cf. sous-extension `methodCollection`) : saisie manuelle, lecture de la carte Vitale, interrogation directe du téléservice INSi, scan d'un code à barre/Datamatrix, lecture RFID. Cette date ne doit pas être confondue avec la date de vérification de l'identité (cf. sous-extension `validationDate`). | Date at which the identity traits or the INS were obtained, regardless of the channel used (see the `methodCollection` sub-extension): manual entry, Vitale card reading, direct query of the INSi teleservice, barcode/Datamatrix scan, RFID reading. This date must not be confused with the identity verification date (see the `validationDate` sub-extension).</t>
+    <t>Date d'obtention des traits d'identité ou du matricule INS | Date the identity traits or the INS identifier were collected</t>
+  </si>
+  <si>
+    <t>Date à laquelle les traits d'identité ou le matricule INS ont été obtenus, quel que soit le canal utilisé (cf. sous-extension `methodCollection`) : saisie manuelle, lecture de la carte Vitale, interrogation directe du téléservice INSi, scan d'un code à barre/Datamatrix, lecture RFID. Cette date ne doit pas être confondue avec la date de vérification de l'identité (cf. sous-extension `validationDate`). | Date at which the identity traits or the INS identifier were obtained, regardless of the channel used (see the `methodCollection` sub-extension): manual entry, Vitale card reading, direct query of the INSi teleservice, barcode/Datamatrix scan, RFID reading. This date must not be confused with the identity verification date (see the `validationDate` sub-extension).</t>
   </si>
   <si>
     <t>Extension.extension:dateCollection.id</t>

</xml_diff>

<commit_message>
Ajoute les invariants RNIV EXI SI 09 sur fr-core-identity-reliability (#335)
Une identité comportant l'attribut douteux (DOUT) ou fictif (FICT) dans
`comment` doit avoir le statut PROV, et FICT/DOUT ne peuvent être cumulés. 2e1b42a3a0db39f646bdaacfe73fae245fb4adcc
</commit_message>
<xml_diff>
--- a/fix/issue-298-identity-status-rniv/ig/StructureDefinition-fr-core-identity-reliability.xlsx
+++ b/fix/issue-298-identity-status-rniv/ig/StructureDefinition-fr-core-identity-reliability.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="172">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-12T13:53:29+00:00</t>
+    <t>2026-08-12T14:08:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -269,7 +269,7 @@
   </si>
   <si>
     <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}</t>
+ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}fr-core-identity-reliability-1:Une identité comportant l'attribut Identité douteuse (DOUT) ou Identité fictive (FICT) dans `comment` doit avoir un statut de confiance (`identityStatus`) égal à Identité provisoire (PROV) [EXI SI 09] {extension('comment').value.coding.exists(code = 'DOUT' or code = 'FICT') implies extension('identityStatus').value.exists(code = 'PROV')}fr-core-identity-reliability-2:Les attributs Identité fictive (FICT) et Identité douteuse (DOUT) ne peuvent être cumulés dans `comment` sur une même identité {extension('comment').value.coding.where(code = 'FICT').exists() implies extension('comment').value.coding.where(code = 'DOUT').empty()}</t>
   </si>
   <si>
     <t>Extension.id</t>
@@ -325,6 +325,10 @@
   </si>
   <si>
     <t>Element.extension</t>
+  </si>
+  <si>
+    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
+ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}</t>
   </si>
   <si>
     <t>Extension.extension:methodCollection</t>
@@ -1319,7 +1323,7 @@
         <v>78</v>
       </c>
       <c r="AJ4" t="s" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="AK4" t="s" s="2">
         <v>90</v>
@@ -1327,13 +1331,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B5" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D5" t="s" s="2">
         <v>78</v>
@@ -1358,10 +1362,10 @@
         <v>93</v>
       </c>
       <c r="L5" t="s" s="2">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M5" t="s" s="2">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -1424,7 +1428,7 @@
         <v>78</v>
       </c>
       <c r="AJ5" t="s" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="AK5" t="s" s="2">
         <v>78</v>
@@ -1432,10 +1436,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
@@ -1535,10 +1539,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
@@ -1567,7 +1571,7 @@
         <v>32</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1630,7 +1634,7 @@
         <v>78</v>
       </c>
       <c r="AJ7" t="s" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="AK7" t="s" s="2">
         <v>78</v>
@@ -1638,10 +1642,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1664,16 +1668,16 @@
         <v>78</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N8" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" t="s" s="2">
@@ -1681,7 +1685,7 @@
       </c>
       <c r="Q8" s="2"/>
       <c r="R8" t="s" s="2">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="S8" t="s" s="2">
         <v>78</v>
@@ -1723,7 +1727,7 @@
         <v>78</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>85</v>
@@ -1738,15 +1742,15 @@
         <v>78</v>
       </c>
       <c r="AK8" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -1769,13 +1773,13 @@
         <v>78</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -1802,11 +1806,11 @@
         <v>78</v>
       </c>
       <c r="X9" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="Y9" s="2"/>
       <c r="Z9" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA9" t="s" s="2">
         <v>78</v>
@@ -1824,7 +1828,7 @@
         <v>78</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>79</v>
@@ -1836,21 +1840,21 @@
         <v>78</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AK9" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B10" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D10" t="s" s="2">
         <v>78</v>
@@ -1875,10 +1879,10 @@
         <v>93</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -1941,7 +1945,7 @@
         <v>78</v>
       </c>
       <c r="AJ10" t="s" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="AK10" t="s" s="2">
         <v>78</v>
@@ -1949,10 +1953,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2052,10 +2056,10 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2084,7 +2088,7 @@
         <v>32</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -2147,7 +2151,7 @@
         <v>78</v>
       </c>
       <c r="AJ12" t="s" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="AK12" t="s" s="2">
         <v>78</v>
@@ -2155,10 +2159,10 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2181,16 +2185,16 @@
         <v>78</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -2198,7 +2202,7 @@
       </c>
       <c r="Q13" s="2"/>
       <c r="R13" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="S13" t="s" s="2">
         <v>78</v>
@@ -2240,7 +2244,7 @@
         <v>78</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>85</v>
@@ -2255,15 +2259,15 @@
         <v>78</v>
       </c>
       <c r="AK13" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2286,13 +2290,13 @@
         <v>78</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2343,7 +2347,7 @@
         <v>78</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>79</v>
@@ -2355,21 +2359,21 @@
         <v>78</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AK14" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B15" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D15" t="s" s="2">
         <v>78</v>
@@ -2394,10 +2398,10 @@
         <v>93</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2460,7 +2464,7 @@
         <v>78</v>
       </c>
       <c r="AJ15" t="s" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="AK15" t="s" s="2">
         <v>78</v>
@@ -2468,10 +2472,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2571,10 +2575,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -2603,7 +2607,7 @@
         <v>32</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -2666,7 +2670,7 @@
         <v>78</v>
       </c>
       <c r="AJ17" t="s" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="AK17" t="s" s="2">
         <v>78</v>
@@ -2674,10 +2678,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -2700,16 +2704,16 @@
         <v>78</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N18" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -2717,7 +2721,7 @@
       </c>
       <c r="Q18" s="2"/>
       <c r="R18" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="S18" t="s" s="2">
         <v>78</v>
@@ -2759,7 +2763,7 @@
         <v>78</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>85</v>
@@ -2774,15 +2778,15 @@
         <v>78</v>
       </c>
       <c r="AK18" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -2805,13 +2809,13 @@
         <v>78</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -2838,11 +2842,11 @@
         <v>78</v>
       </c>
       <c r="X19" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Y19" s="2"/>
       <c r="Z19" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="AA19" t="s" s="2">
         <v>78</v>
@@ -2860,7 +2864,7 @@
         <v>78</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>79</v>
@@ -2872,21 +2876,21 @@
         <v>78</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B20" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C20" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D20" t="s" s="2">
         <v>78</v>
@@ -2911,10 +2915,10 @@
         <v>93</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -2977,7 +2981,7 @@
         <v>78</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="AK20" t="s" s="2">
         <v>78</v>
@@ -2985,10 +2989,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3088,10 +3092,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3120,7 +3124,7 @@
         <v>32</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -3183,7 +3187,7 @@
         <v>78</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="AK22" t="s" s="2">
         <v>78</v>
@@ -3191,10 +3195,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3217,16 +3221,16 @@
         <v>78</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -3234,7 +3238,7 @@
       </c>
       <c r="Q23" s="2"/>
       <c r="R23" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="S23" t="s" s="2">
         <v>78</v>
@@ -3276,7 +3280,7 @@
         <v>78</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>85</v>
@@ -3291,15 +3295,15 @@
         <v>78</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3322,13 +3326,13 @@
         <v>78</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -3355,11 +3359,11 @@
         <v>78</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="Y24" s="2"/>
       <c r="Z24" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>78</v>
@@ -3377,7 +3381,7 @@
         <v>78</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>79</v>
@@ -3389,21 +3393,21 @@
         <v>78</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B25" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C25" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D25" t="s" s="2">
         <v>78</v>
@@ -3428,10 +3432,10 @@
         <v>93</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -3494,7 +3498,7 @@
         <v>78</v>
       </c>
       <c r="AJ25" t="s" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="AK25" t="s" s="2">
         <v>78</v>
@@ -3502,10 +3506,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -3605,10 +3609,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -3637,7 +3641,7 @@
         <v>32</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -3700,7 +3704,7 @@
         <v>78</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="AK27" t="s" s="2">
         <v>78</v>
@@ -3708,10 +3712,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -3734,16 +3738,16 @@
         <v>78</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -3751,7 +3755,7 @@
       </c>
       <c r="Q28" s="2"/>
       <c r="R28" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="S28" t="s" s="2">
         <v>78</v>
@@ -3793,7 +3797,7 @@
         <v>78</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>85</v>
@@ -3808,15 +3812,15 @@
         <v>78</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -3839,13 +3843,13 @@
         <v>78</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -3896,7 +3900,7 @@
         <v>78</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>79</v>
@@ -3908,21 +3912,21 @@
         <v>78</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B30" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C30" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D30" t="s" s="2">
         <v>78</v>
@@ -3947,10 +3951,10 @@
         <v>93</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -4013,7 +4017,7 @@
         <v>78</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="AK30" t="s" s="2">
         <v>78</v>
@@ -4021,10 +4025,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4124,10 +4128,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -4156,7 +4160,7 @@
         <v>32</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -4219,7 +4223,7 @@
         <v>78</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="AK32" t="s" s="2">
         <v>78</v>
@@ -4227,10 +4231,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -4253,16 +4257,16 @@
         <v>78</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
@@ -4270,7 +4274,7 @@
       </c>
       <c r="Q33" s="2"/>
       <c r="R33" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S33" t="s" s="2">
         <v>78</v>
@@ -4312,7 +4316,7 @@
         <v>78</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>85</v>
@@ -4327,15 +4331,15 @@
         <v>78</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -4358,13 +4362,13 @@
         <v>78</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -4391,11 +4395,11 @@
         <v>78</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Y34" s="2"/>
       <c r="Z34" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>78</v>
@@ -4413,7 +4417,7 @@
         <v>78</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>79</v>
@@ -4425,18 +4429,18 @@
         <v>78</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -4459,16 +4463,16 @@
         <v>78</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -4518,7 +4522,7 @@
         <v>78</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>85</v>
@@ -4533,15 +4537,15 @@
         <v>78</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -4564,13 +4568,13 @@
         <v>78</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -4621,7 +4625,7 @@
         <v>78</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>79</v>
@@ -4633,10 +4637,10 @@
         <v>78</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>